<commit_message>
Update to write custom rates and hpos
</commit_message>
<xml_diff>
--- a/Assets/HPOs.xlsx
+++ b/Assets/HPOs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AI-Operator\HPO-Package-Builder\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0538505-7D14-4C17-8041-5D6290286DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F49D7E-33D3-4523-B3E5-ED9EF72DF8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{243C507C-E199-47F9-83A6-533C684884E7}"/>
+    <workbookView xWindow="22932" yWindow="-1524" windowWidth="23256" windowHeight="12456" xr2:uid="{243C507C-E199-47F9-83A6-533C684884E7}"/>
   </bookViews>
   <sheets>
     <sheet name="HPOs" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>College Football - 2026-2027</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t>World Cup</t>
+  </si>
+  <si>
+    <t>Custom HPO</t>
   </si>
 </sst>
 </file>
@@ -157,8 +160,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CB179BAC-9D1B-405D-B7F1-DD277E5752CA}" name="Table1" displayName="Table1" ref="A1:B11" totalsRowShown="0">
-  <autoFilter ref="A1:B11" xr:uid="{CB179BAC-9D1B-405D-B7F1-DD277E5752CA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CB179BAC-9D1B-405D-B7F1-DD277E5752CA}" name="Table1" displayName="Table1" ref="A1:B12" totalsRowShown="0">
+  <autoFilter ref="A1:B12" xr:uid="{CB179BAC-9D1B-405D-B7F1-DD277E5752CA}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{CEB0B6A3-7923-4935-9127-B5B310F76137}" name="HPOs"/>
     <tableColumn id="2" xr3:uid="{1EFF6380-28C5-4462-A6CC-46063A6A573C}" name="Sport"/>
@@ -484,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B724845-B2D3-47DE-B694-66454D902E75}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
@@ -579,6 +582,14 @@
         <v>21</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>